<commit_message>
improve compatibility with stare scans
</commit_message>
<xml_diff>
--- a/configs/config_g3p3_a0.xlsx
+++ b/configs/config_g3p3_a0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SLETIZIA\OneDrive - NREL\Desktop\Main\G3P3\g3p3_lidar_processing\configs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aabraha2\Documents\G3P3\Codes\g3p3_lidar_processing\configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CF25EC-4CB5-4F43-9528-EFB655ACA100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{692D280B-D9F9-4C04-A5D8-49917516723E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1596" yWindow="348" windowWidth="21600" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
   <si>
     <t>a0</t>
   </si>
@@ -63,6 +63,12 @@
   </si>
   <si>
     <t>257_\d{8}_\d{2}.hpl</t>
+  </si>
+  <si>
+    <t>327_\d{8}_\d{2}.hpl</t>
+  </si>
+  <si>
+    <t>g3p3</t>
   </si>
 </sst>
 </file>
@@ -506,7 +512,9 @@
       <c r="C1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
     </row>
@@ -520,7 +528,9 @@
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
@@ -534,7 +544,9 @@
       <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
@@ -548,7 +560,9 @@
       <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
@@ -562,7 +576,9 @@
       <c r="C5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
     </row>

</xml_diff>